<commit_message>
Add physical-language alignment study and consolidate H16 experiments
</commit_message>
<xml_diff>
--- a/outputs/final_h16/formal_comparison_subset_with_fm.xlsx
+++ b/outputs/final_h16/formal_comparison_subset_with_fm.xlsx
@@ -120,10 +120,10 @@
     <xf numFmtId="164" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="5" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -589,7 +589,7 @@
     <row r="2" ht="34" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>15 min resolution; L96 (24 h) to H16 (4 h); chronological 70%/15%/15%; seed 2026. Metrics use each station's native target scale; MBE = prediction - observation. Ours (PSRC+FM) uses validation-locked adapters and the single test unblinding on 2026-09-16, with no test-based reselection. Ours improves test RMSE on 3 of 4 stations; the real prior beats the shuffled-prior control on all 4.</t>
+          <t>15 min resolution; L96 (24 h) to H16 (4 h); chronological 70%/15%/15%; seed 2026. Metrics use each station's native target scale; MSE = mean squared error, RMSE = sqrt(MSE). LSTM/GRU are locked sensitivity configurations, not public-default baselines.</t>
         </is>
       </c>
     </row>
@@ -710,7 +710,7 @@
       <c r="BB3" s="3" t="n"/>
       <c r="BC3" s="3" t="inlineStr">
         <is>
-          <t>LSTM</t>
+          <t>LSTM (h128, 3L, d0.3)</t>
         </is>
       </c>
       <c r="BD3" s="3" t="n"/>
@@ -718,7 +718,7 @@
       <c r="BF3" s="3" t="n"/>
       <c r="BG3" s="3" t="inlineStr">
         <is>
-          <t>GRU</t>
+          <t>GRU (h64, 3L, d0.3)</t>
         </is>
       </c>
       <c r="BH3" s="3" t="n"/>
@@ -764,7 +764,7 @@
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>MBE</t>
+          <t>MSE</t>
         </is>
       </c>
       <c r="F4" s="3" t="inlineStr">
@@ -784,7 +784,7 @@
       </c>
       <c r="I4" s="3" t="inlineStr">
         <is>
-          <t>MBE</t>
+          <t>MSE</t>
         </is>
       </c>
       <c r="J4" s="3" t="inlineStr">
@@ -804,7 +804,7 @@
       </c>
       <c r="M4" s="3" t="inlineStr">
         <is>
-          <t>MBE</t>
+          <t>MSE</t>
         </is>
       </c>
       <c r="N4" s="3" t="inlineStr">
@@ -824,7 +824,7 @@
       </c>
       <c r="Q4" s="3" t="inlineStr">
         <is>
-          <t>MBE</t>
+          <t>MSE</t>
         </is>
       </c>
       <c r="R4" s="3" t="inlineStr">
@@ -844,7 +844,7 @@
       </c>
       <c r="U4" s="3" t="inlineStr">
         <is>
-          <t>MBE</t>
+          <t>MSE</t>
         </is>
       </c>
       <c r="V4" s="3" t="inlineStr">
@@ -864,7 +864,7 @@
       </c>
       <c r="Y4" s="3" t="inlineStr">
         <is>
-          <t>MBE</t>
+          <t>MSE</t>
         </is>
       </c>
       <c r="Z4" s="3" t="inlineStr">
@@ -884,7 +884,7 @@
       </c>
       <c r="AC4" s="3" t="inlineStr">
         <is>
-          <t>MBE</t>
+          <t>MSE</t>
         </is>
       </c>
       <c r="AD4" s="3" t="inlineStr">
@@ -904,7 +904,7 @@
       </c>
       <c r="AG4" s="3" t="inlineStr">
         <is>
-          <t>MBE</t>
+          <t>MSE</t>
         </is>
       </c>
       <c r="AH4" s="3" t="inlineStr">
@@ -924,7 +924,7 @@
       </c>
       <c r="AK4" s="3" t="inlineStr">
         <is>
-          <t>MBE</t>
+          <t>MSE</t>
         </is>
       </c>
       <c r="AL4" s="3" t="inlineStr">
@@ -944,7 +944,7 @@
       </c>
       <c r="AO4" s="3" t="inlineStr">
         <is>
-          <t>MBE</t>
+          <t>MSE</t>
         </is>
       </c>
       <c r="AP4" s="3" t="inlineStr">
@@ -964,7 +964,7 @@
       </c>
       <c r="AS4" s="3" t="inlineStr">
         <is>
-          <t>MBE</t>
+          <t>MSE</t>
         </is>
       </c>
       <c r="AT4" s="3" t="inlineStr">
@@ -984,7 +984,7 @@
       </c>
       <c r="AW4" s="3" t="inlineStr">
         <is>
-          <t>MBE</t>
+          <t>MSE</t>
         </is>
       </c>
       <c r="AX4" s="3" t="inlineStr">
@@ -1004,7 +1004,7 @@
       </c>
       <c r="BA4" s="3" t="inlineStr">
         <is>
-          <t>MBE</t>
+          <t>MSE</t>
         </is>
       </c>
       <c r="BB4" s="3" t="inlineStr">
@@ -1024,7 +1024,7 @@
       </c>
       <c r="BE4" s="3" t="inlineStr">
         <is>
-          <t>MBE</t>
+          <t>MSE</t>
         </is>
       </c>
       <c r="BF4" s="3" t="inlineStr">
@@ -1044,7 +1044,7 @@
       </c>
       <c r="BI4" s="3" t="inlineStr">
         <is>
-          <t>MBE</t>
+          <t>MSE</t>
         </is>
       </c>
       <c r="BJ4" s="3" t="inlineStr">
@@ -1064,7 +1064,7 @@
       </c>
       <c r="BM4" s="3" t="inlineStr">
         <is>
-          <t>MBE</t>
+          <t>MSE</t>
         </is>
       </c>
       <c r="BN4" s="3" t="inlineStr">
@@ -1084,7 +1084,7 @@
       </c>
       <c r="BQ4" s="3" t="inlineStr">
         <is>
-          <t>MBE</t>
+          <t>MSE</t>
         </is>
       </c>
       <c r="BR4" s="3" t="inlineStr">
@@ -1104,7 +1104,7 @@
       </c>
       <c r="BU4" s="3" t="inlineStr">
         <is>
-          <t>MBE</t>
+          <t>MSE</t>
         </is>
       </c>
       <c r="BV4" s="3" t="inlineStr">
@@ -1130,214 +1130,214 @@
       <c r="D5" s="5" t="n">
         <v>0.1286411575529365</v>
       </c>
-      <c r="E5" s="6" t="n">
-        <v>-0.00694702990903869</v>
+      <c r="E5" s="5" t="n">
+        <v>0.08476488220272187</v>
       </c>
       <c r="F5" s="5" t="n">
         <v>0.9484481532970693</v>
       </c>
-      <c r="G5" s="7" t="n">
+      <c r="G5" s="6" t="n">
         <v>0.2897142913896061</v>
       </c>
-      <c r="H5" s="7" t="n">
+      <c r="H5" s="6" t="n">
         <v>0.1258303423559397</v>
       </c>
-      <c r="I5" s="7" t="n">
-        <v>-0.0002665334964434959</v>
-      </c>
-      <c r="J5" s="7" t="n">
+      <c r="I5" s="6" t="n">
+        <v>0.08393437063538162</v>
+      </c>
+      <c r="J5" s="6" t="n">
         <v>0.9489532493214128</v>
       </c>
-      <c r="K5" s="6" t="n">
+      <c r="K5" s="7" t="n">
         <v>0.321479362926304</v>
       </c>
-      <c r="L5" s="6" t="n">
+      <c r="L5" s="7" t="n">
         <v>0.1494558522787549</v>
       </c>
-      <c r="M5" s="6" t="n">
-        <v>0.02807145895822704</v>
-      </c>
-      <c r="N5" s="6" t="n">
+      <c r="M5" s="7" t="n">
+        <v>0.1033489807875023</v>
+      </c>
+      <c r="N5" s="7" t="n">
         <v>0.9371457769301264</v>
       </c>
-      <c r="O5" s="6" t="n">
+      <c r="O5" s="7" t="n">
         <v>0.3041312591084534</v>
       </c>
-      <c r="P5" s="6" t="n">
+      <c r="P5" s="7" t="n">
         <v>0.1448192533228003</v>
       </c>
-      <c r="Q5" s="6" t="n">
-        <v>0.01894073520444747</v>
-      </c>
-      <c r="R5" s="6" t="n">
+      <c r="Q5" s="7" t="n">
+        <v>0.09249582276689322</v>
+      </c>
+      <c r="R5" s="7" t="n">
         <v>0.9437463917600157</v>
       </c>
-      <c r="S5" s="6" t="n">
+      <c r="S5" s="7" t="n">
         <v>0.3235817914628595</v>
       </c>
-      <c r="T5" s="6" t="n">
+      <c r="T5" s="7" t="n">
         <v>0.1681565203835893</v>
       </c>
-      <c r="U5" s="6" t="n">
-        <v>-0.01354318249595851</v>
-      </c>
-      <c r="V5" s="6" t="n">
+      <c r="U5" s="7" t="n">
+        <v>0.1047051757663135</v>
+      </c>
+      <c r="V5" s="7" t="n">
         <v>0.9363209736173611</v>
       </c>
-      <c r="W5" s="6" t="n">
+      <c r="W5" s="7" t="n">
         <v>0.3159967545661116</v>
       </c>
-      <c r="X5" s="6" t="n">
+      <c r="X5" s="7" t="n">
         <v>0.1579615265199842</v>
       </c>
-      <c r="Y5" s="6" t="n">
-        <v>0.01380849567297425</v>
-      </c>
-      <c r="Z5" s="6" t="n">
+      <c r="Y5" s="7" t="n">
+        <v>0.09985394889631537</v>
+      </c>
+      <c r="Z5" s="7" t="n">
         <v>0.9392713664855441</v>
       </c>
-      <c r="AA5" s="6" t="n">
+      <c r="AA5" s="7" t="n">
         <v>0.350453244685843</v>
       </c>
-      <c r="AB5" s="6" t="n">
+      <c r="AB5" s="7" t="n">
         <v>0.2302267456847937</v>
       </c>
-      <c r="AC5" s="6" t="n">
-        <v>0.0641714950327358</v>
-      </c>
-      <c r="AD5" s="6" t="n">
+      <c r="AC5" s="7" t="n">
+        <v>0.1228174767108353</v>
+      </c>
+      <c r="AD5" s="7" t="n">
         <v>0.9253055325825199</v>
       </c>
-      <c r="AE5" s="6" t="n">
+      <c r="AE5" s="7" t="n">
         <v>0.3318136548095944</v>
       </c>
-      <c r="AF5" s="6" t="n">
+      <c r="AF5" s="7" t="n">
         <v>0.1567716505994267</v>
       </c>
-      <c r="AG5" s="6" t="n">
-        <v>0.02205336342930977</v>
-      </c>
-      <c r="AH5" s="6" t="n">
+      <c r="AG5" s="7" t="n">
+        <v>0.1101003015181007</v>
+      </c>
+      <c r="AH5" s="7" t="n">
         <v>0.9330397952747309</v>
       </c>
-      <c r="AI5" s="6" t="n">
+      <c r="AI5" s="7" t="n">
         <v>0.3314855861776914</v>
       </c>
-      <c r="AJ5" s="6" t="n">
+      <c r="AJ5" s="7" t="n">
         <v>0.1605179710956233</v>
       </c>
-      <c r="AK5" s="6" t="n">
-        <v>0.0327112979158086</v>
-      </c>
-      <c r="AL5" s="6" t="n">
+      <c r="AK5" s="7" t="n">
+        <v>0.1098826938435676</v>
+      </c>
+      <c r="AL5" s="7" t="n">
         <v>0.9331721387309759</v>
       </c>
-      <c r="AM5" s="6" t="n">
+      <c r="AM5" s="7" t="n">
         <v>0.3010395270456998</v>
       </c>
-      <c r="AN5" s="6" t="n">
+      <c r="AN5" s="7" t="n">
         <v>0.1377292612525472</v>
       </c>
-      <c r="AO5" s="6" t="n">
-        <v>-0.003676748451694571</v>
-      </c>
-      <c r="AP5" s="6" t="n">
+      <c r="AO5" s="7" t="n">
+        <v>0.0906247968438986</v>
+      </c>
+      <c r="AP5" s="7" t="n">
         <v>0.9448843021664592</v>
       </c>
-      <c r="AQ5" s="6" t="n">
+      <c r="AQ5" s="7" t="n">
         <v>0.3025345034148401</v>
       </c>
-      <c r="AR5" s="6" t="n">
+      <c r="AR5" s="7" t="n">
         <v>0.137429680605658</v>
       </c>
-      <c r="AS5" s="6" t="n">
-        <v>-0.004438834804926809</v>
-      </c>
-      <c r="AT5" s="6" t="n">
+      <c r="AS5" s="7" t="n">
+        <v>0.09152712575646388</v>
+      </c>
+      <c r="AT5" s="7" t="n">
         <v>0.9443355286582871</v>
       </c>
-      <c r="AU5" s="6" t="n">
+      <c r="AU5" s="7" t="n">
         <v>0.3047627604745357</v>
       </c>
-      <c r="AV5" s="6" t="n">
+      <c r="AV5" s="7" t="n">
         <v>0.1605678936569842</v>
       </c>
-      <c r="AW5" s="6" t="n">
-        <v>0.04129668529962</v>
-      </c>
-      <c r="AX5" s="6" t="n">
+      <c r="AW5" s="7" t="n">
+        <v>0.09288034017205919</v>
+      </c>
+      <c r="AX5" s="7" t="n">
         <v>0.9435125380483063</v>
       </c>
-      <c r="AY5" s="6" t="n">
+      <c r="AY5" s="7" t="n">
         <v>0.3160656651469466</v>
       </c>
-      <c r="AZ5" s="6" t="n">
+      <c r="AZ5" s="7" t="n">
         <v>0.1628060257869335</v>
       </c>
-      <c r="BA5" s="6" t="n">
-        <v>0.04367169318931059</v>
-      </c>
-      <c r="BB5" s="6" t="n">
+      <c r="BA5" s="7" t="n">
+        <v>0.09989750468478178</v>
+      </c>
+      <c r="BB5" s="7" t="n">
         <v>0.9392448769621506</v>
       </c>
-      <c r="BC5" s="6" t="n">
-        <v>0.3423042147955348</v>
-      </c>
-      <c r="BD5" s="6" t="n">
-        <v>0.1776458453566785</v>
-      </c>
-      <c r="BE5" s="6" t="n">
-        <v>0.1047482420099436</v>
-      </c>
-      <c r="BF5" s="6" t="n">
-        <v>0.9287388613002902</v>
-      </c>
-      <c r="BG5" s="6" t="n">
-        <v>0.3270403413865789</v>
-      </c>
-      <c r="BH5" s="6" t="n">
-        <v>0.1649215518640358</v>
-      </c>
-      <c r="BI5" s="6" t="n">
-        <v>0.08829006294450231</v>
-      </c>
-      <c r="BJ5" s="6" t="n">
-        <v>0.9349524536241935</v>
-      </c>
-      <c r="BK5" s="6" t="n">
+      <c r="BC5" s="7" t="n">
+        <v>0.3456709841600824</v>
+      </c>
+      <c r="BD5" s="7" t="n">
+        <v>0.1707549705470336</v>
+      </c>
+      <c r="BE5" s="7" t="n">
+        <v>0.1194884292901999</v>
+      </c>
+      <c r="BF5" s="7" t="n">
+        <v>0.9273301746021354</v>
+      </c>
+      <c r="BG5" s="7" t="n">
+        <v>0.3570098392867278</v>
+      </c>
+      <c r="BH5" s="7" t="n">
+        <v>0.1826681691831938</v>
+      </c>
+      <c r="BI5" s="7" t="n">
+        <v>0.1274560253475352</v>
+      </c>
+      <c r="BJ5" s="7" t="n">
+        <v>0.9224844852097253</v>
+      </c>
+      <c r="BK5" s="7" t="n">
         <v>0.3302271523408281</v>
       </c>
-      <c r="BL5" s="6" t="n">
+      <c r="BL5" s="7" t="n">
         <v>0.1774173178073225</v>
       </c>
-      <c r="BM5" s="6" t="n">
-        <v>0.05845102062314993</v>
-      </c>
-      <c r="BN5" s="6" t="n">
+      <c r="BM5" s="7" t="n">
+        <v>0.1090499721431325</v>
+      </c>
+      <c r="BN5" s="7" t="n">
         <v>0.9336785789020879</v>
       </c>
-      <c r="BO5" s="6" t="n">
+      <c r="BO5" s="7" t="n">
         <v>0.9602006283445177</v>
       </c>
-      <c r="BP5" s="6" t="n">
+      <c r="BP5" s="7" t="n">
         <v>0.5734639102279436</v>
       </c>
-      <c r="BQ5" s="5" t="n">
-        <v>-0.003651163009907553</v>
-      </c>
-      <c r="BR5" s="6" t="n">
+      <c r="BQ5" s="7" t="n">
+        <v>0.9219852466732066</v>
+      </c>
+      <c r="BR5" s="7" t="n">
         <v>0.4392720090710555</v>
       </c>
-      <c r="BS5" s="6" t="n">
+      <c r="BS5" s="7" t="n">
         <v>0.4573214763492157</v>
       </c>
-      <c r="BT5" s="6" t="n">
+      <c r="BT5" s="7" t="n">
         <v>0.1752165732063827</v>
       </c>
-      <c r="BU5" s="6" t="n">
-        <v>-0.009021839725515313</v>
-      </c>
-      <c r="BV5" s="6" t="n">
+      <c r="BU5" s="7" t="n">
+        <v>0.2091429327302263</v>
+      </c>
+      <c r="BV5" s="7" t="n">
         <v>0.8728045845527789</v>
       </c>
     </row>
@@ -1355,217 +1355,217 @@
       <c r="C6" s="5" t="n">
         <v>0.7388191954047842</v>
       </c>
-      <c r="D6" s="6" t="n">
+      <c r="D6" s="7" t="n">
         <v>0.4038139184202177</v>
       </c>
-      <c r="E6" s="6" t="n">
-        <v>-0.005709139409897456</v>
+      <c r="E6" s="5" t="n">
+        <v>0.5458538034985728</v>
       </c>
       <c r="F6" s="5" t="n">
         <v>0.9353890447570046</v>
       </c>
-      <c r="G6" s="7" t="n">
-        <v>0.7312909762378148</v>
-      </c>
-      <c r="H6" s="7" t="n">
-        <v>0.3693376633213977</v>
+      <c r="G6" s="6" t="n">
+        <v>0.7298797086128039</v>
+      </c>
+      <c r="H6" s="6" t="n">
+        <v>0.3645763346962462</v>
       </c>
       <c r="I6" s="6" t="n">
-        <v>-0.006287771875430512</v>
-      </c>
-      <c r="J6" s="7" t="n">
-        <v>0.9366990467539447</v>
-      </c>
-      <c r="K6" s="6" t="n">
+        <v>0.5327243890447115</v>
+      </c>
+      <c r="J6" s="6" t="n">
+        <v>0.9369431312252275</v>
+      </c>
+      <c r="K6" s="7" t="n">
         <v>0.7958735101539998</v>
       </c>
-      <c r="L6" s="6" t="n">
+      <c r="L6" s="7" t="n">
         <v>0.4104786037439699</v>
       </c>
-      <c r="M6" s="6" t="n">
-        <v>0.06539757927799281</v>
-      </c>
-      <c r="N6" s="6" t="n">
+      <c r="M6" s="7" t="n">
+        <v>0.6334146441648487</v>
+      </c>
+      <c r="N6" s="7" t="n">
         <v>0.9250247502864567</v>
       </c>
-      <c r="O6" s="6" t="n">
+      <c r="O6" s="7" t="n">
         <v>0.7697433727672575</v>
       </c>
       <c r="P6" s="5" t="n">
         <v>0.3704294834261007</v>
       </c>
-      <c r="Q6" s="6" t="n">
-        <v>0.07609527495926698</v>
-      </c>
-      <c r="R6" s="6" t="n">
+      <c r="Q6" s="7" t="n">
+        <v>0.5925048599191131</v>
+      </c>
+      <c r="R6" s="7" t="n">
         <v>0.9298671095811258</v>
       </c>
-      <c r="S6" s="6" t="n">
+      <c r="S6" s="7" t="n">
         <v>0.8740008464623079</v>
       </c>
-      <c r="T6" s="6" t="n">
+      <c r="T6" s="7" t="n">
         <v>0.5224367065056674</v>
       </c>
-      <c r="U6" s="6" t="n">
-        <v>-0.01250395916986872</v>
-      </c>
-      <c r="V6" s="6" t="n">
+      <c r="U6" s="7" t="n">
+        <v>0.7638774796168307</v>
+      </c>
+      <c r="V6" s="7" t="n">
         <v>0.9095822849812125</v>
       </c>
-      <c r="W6" s="6" t="n">
+      <c r="W6" s="7" t="n">
         <v>0.7789428089104529</v>
       </c>
-      <c r="X6" s="6" t="n">
+      <c r="X6" s="7" t="n">
         <v>0.3812202844414812</v>
       </c>
-      <c r="Y6" s="6" t="n">
-        <v>0.1027829411874508</v>
-      </c>
-      <c r="Z6" s="6" t="n">
+      <c r="Y6" s="7" t="n">
+        <v>0.6067518995533063</v>
+      </c>
+      <c r="Z6" s="7" t="n">
         <v>0.9281807334228027</v>
       </c>
-      <c r="AA6" s="6" t="n">
+      <c r="AA6" s="7" t="n">
         <v>0.8521951770106725</v>
       </c>
-      <c r="AB6" s="6" t="n">
+      <c r="AB6" s="7" t="n">
         <v>0.6110119829863081</v>
       </c>
-      <c r="AC6" s="6" t="n">
-        <v>0.06521457315692647</v>
-      </c>
-      <c r="AD6" s="6" t="n">
+      <c r="AC6" s="7" t="n">
+        <v>0.7262366197202514</v>
+      </c>
+      <c r="AD6" s="7" t="n">
         <v>0.914037712237555</v>
       </c>
-      <c r="AE6" s="6" t="n">
+      <c r="AE6" s="7" t="n">
         <v>0.7974374785119308</v>
       </c>
-      <c r="AF6" s="6" t="n">
+      <c r="AF6" s="7" t="n">
         <v>0.4004954741197432</v>
       </c>
-      <c r="AG6" s="6" t="n">
-        <v>0.03681140399003567</v>
-      </c>
-      <c r="AH6" s="6" t="n">
+      <c r="AG6" s="7" t="n">
+        <v>0.6359065321354661</v>
+      </c>
+      <c r="AH6" s="7" t="n">
         <v>0.9247297935395985</v>
       </c>
-      <c r="AI6" s="6" t="n">
+      <c r="AI6" s="7" t="n">
         <v>0.8454068500976658</v>
       </c>
-      <c r="AJ6" s="6" t="n">
+      <c r="AJ6" s="7" t="n">
         <v>0.4312824667309331</v>
       </c>
-      <c r="AK6" s="5" t="n">
-        <v>-0.001009587531884746</v>
-      </c>
-      <c r="AL6" s="6" t="n">
+      <c r="AK6" s="7" t="n">
+        <v>0.7147127421920572</v>
+      </c>
+      <c r="AL6" s="7" t="n">
         <v>0.9154017564750921</v>
       </c>
-      <c r="AM6" s="6" t="n">
+      <c r="AM6" s="7" t="n">
         <v>0.7774884210743088</v>
       </c>
-      <c r="AN6" s="6" t="n">
+      <c r="AN6" s="7" t="n">
         <v>0.3915632334055896</v>
       </c>
-      <c r="AO6" s="6" t="n">
-        <v>0.03580489575241635</v>
-      </c>
-      <c r="AP6" s="6" t="n">
+      <c r="AO6" s="7" t="n">
+        <v>0.6044882449046217</v>
+      </c>
+      <c r="AP6" s="7" t="n">
         <v>0.9284486749270192</v>
       </c>
-      <c r="AQ6" s="6" t="n">
+      <c r="AQ6" s="7" t="n">
         <v>0.7547368403949566</v>
       </c>
-      <c r="AR6" s="6" t="n">
+      <c r="AR6" s="7" t="n">
         <v>0.3705520836789533</v>
       </c>
-      <c r="AS6" s="6" t="n">
-        <v>0.003949134833280936</v>
-      </c>
-      <c r="AT6" s="6" t="n">
+      <c r="AS6" s="7" t="n">
+        <v>0.5696276982493622</v>
+      </c>
+      <c r="AT6" s="7" t="n">
         <v>0.9325750054669056</v>
       </c>
-      <c r="AU6" s="6" t="n">
+      <c r="AU6" s="7" t="n">
         <v>0.7822109435625039</v>
       </c>
-      <c r="AV6" s="6" t="n">
+      <c r="AV6" s="7" t="n">
         <v>0.4094125778213651</v>
       </c>
-      <c r="AW6" s="6" t="n">
-        <v>-0.03532406143850002</v>
-      </c>
-      <c r="AX6" s="6" t="n">
+      <c r="AW6" s="7" t="n">
+        <v>0.6118539602289426</v>
+      </c>
+      <c r="AX6" s="7" t="n">
         <v>0.927576818946348</v>
       </c>
-      <c r="AY6" s="6" t="n">
+      <c r="AY6" s="7" t="n">
         <v>0.8075224874504936</v>
       </c>
-      <c r="AZ6" s="6" t="n">
+      <c r="AZ6" s="7" t="n">
         <v>0.4260618703518039</v>
       </c>
-      <c r="BA6" s="6" t="n">
-        <v>0.04942095600268308</v>
-      </c>
-      <c r="BB6" s="6" t="n">
+      <c r="BA6" s="7" t="n">
+        <v>0.6520925677382325</v>
+      </c>
+      <c r="BB6" s="7" t="n">
         <v>0.9228139046785354</v>
       </c>
-      <c r="BC6" s="6" t="n">
-        <v>0.8347060913868016</v>
-      </c>
-      <c r="BD6" s="6" t="n">
-        <v>0.4080534095523621</v>
-      </c>
-      <c r="BE6" s="6" t="n">
-        <v>0.07589336890281539</v>
-      </c>
-      <c r="BF6" s="6" t="n">
-        <v>0.9175298115798254</v>
-      </c>
-      <c r="BG6" s="6" t="n">
-        <v>0.7974338014109333</v>
-      </c>
-      <c r="BH6" s="6" t="n">
-        <v>0.3875301397852959</v>
-      </c>
-      <c r="BI6" s="6" t="n">
-        <v>0.02739107967261647</v>
-      </c>
-      <c r="BJ6" s="6" t="n">
-        <v>0.9247304877018886</v>
-      </c>
-      <c r="BK6" s="6" t="n">
+      <c r="BC6" s="7" t="n">
+        <v>0.8820166443314287</v>
+      </c>
+      <c r="BD6" s="7" t="n">
+        <v>0.4339120685635658</v>
+      </c>
+      <c r="BE6" s="7" t="n">
+        <v>0.777953360877674</v>
+      </c>
+      <c r="BF6" s="7" t="n">
+        <v>0.9079161682878396</v>
+      </c>
+      <c r="BG6" s="7" t="n">
+        <v>0.8042251155565121</v>
+      </c>
+      <c r="BH6" s="7" t="n">
+        <v>0.4101923270899676</v>
+      </c>
+      <c r="BI6" s="7" t="n">
+        <v>0.6467780364918853</v>
+      </c>
+      <c r="BJ6" s="7" t="n">
+        <v>0.9234429686115783</v>
+      </c>
+      <c r="BK6" s="7" t="n">
         <v>0.8026796028267282</v>
       </c>
-      <c r="BL6" s="6" t="n">
+      <c r="BL6" s="7" t="n">
         <v>0.4437564999675101</v>
       </c>
-      <c r="BM6" s="6" t="n">
-        <v>0.014982635048107</v>
-      </c>
-      <c r="BN6" s="6" t="n">
+      <c r="BM6" s="7" t="n">
+        <v>0.6442945447940742</v>
+      </c>
+      <c r="BN6" s="7" t="n">
         <v>0.9237369315186885</v>
       </c>
-      <c r="BO6" s="6" t="n">
+      <c r="BO6" s="7" t="n">
         <v>2.165023270699363</v>
       </c>
-      <c r="BP6" s="6" t="n">
+      <c r="BP6" s="7" t="n">
         <v>1.246694674080566</v>
       </c>
-      <c r="BQ6" s="6" t="n">
-        <v>-0.01567015919754333</v>
-      </c>
-      <c r="BR6" s="6" t="n">
+      <c r="BQ6" s="7" t="n">
+        <v>4.687325762669768</v>
+      </c>
+      <c r="BR6" s="7" t="n">
         <v>0.4451763583580356</v>
       </c>
-      <c r="BS6" s="6" t="n">
+      <c r="BS6" s="7" t="n">
         <v>1.067132514083138</v>
       </c>
-      <c r="BT6" s="6" t="n">
+      <c r="BT6" s="7" t="n">
         <v>0.4661126929411851</v>
       </c>
       <c r="BU6" s="7" t="n">
-        <v>-0.0002786930468357129</v>
-      </c>
-      <c r="BV6" s="6" t="n">
+        <v>1.138771802613399</v>
+      </c>
+      <c r="BV6" s="7" t="n">
         <v>0.8652072523832256</v>
       </c>
     </row>
@@ -1580,220 +1580,220 @@
           <t>L96-H16</t>
         </is>
       </c>
-      <c r="C7" s="6" t="n">
+      <c r="C7" s="5" t="n">
         <v>1.67550566661812</v>
       </c>
-      <c r="D7" s="6" t="n">
+      <c r="D7" s="5" t="n">
         <v>0.885519092647951</v>
       </c>
-      <c r="E7" s="6" t="n">
-        <v>0.07808133659629743</v>
-      </c>
-      <c r="F7" s="6" t="n">
+      <c r="E7" s="5" t="n">
+        <v>2.807319238869431</v>
+      </c>
+      <c r="F7" s="5" t="n">
         <v>0.8875405806968881</v>
       </c>
-      <c r="G7" s="7" t="n">
+      <c r="G7" s="6" t="n">
         <v>1.645698707509013</v>
       </c>
-      <c r="H7" s="7" t="n">
+      <c r="H7" s="6" t="n">
         <v>0.8415841307429187</v>
       </c>
       <c r="I7" s="6" t="n">
-        <v>0.02075091371458484</v>
-      </c>
-      <c r="J7" s="7" t="n">
+        <v>2.708324235896837</v>
+      </c>
+      <c r="J7" s="6" t="n">
         <v>0.891506257415825</v>
       </c>
-      <c r="K7" s="6" t="n">
+      <c r="K7" s="7" t="n">
         <v>1.751857158830392</v>
       </c>
-      <c r="L7" s="6" t="n">
+      <c r="L7" s="7" t="n">
         <v>0.9209939041792786</v>
       </c>
-      <c r="M7" s="6" t="n">
-        <v>-0.04662548342549326</v>
-      </c>
-      <c r="N7" s="6" t="n">
+      <c r="M7" s="7" t="n">
+        <v>3.069003504945292</v>
+      </c>
+      <c r="N7" s="7" t="n">
         <v>0.8770576757973714</v>
       </c>
-      <c r="O7" s="6" t="n">
+      <c r="O7" s="7" t="n">
         <v>1.711196529730524</v>
       </c>
-      <c r="P7" s="6" t="n">
+      <c r="P7" s="7" t="n">
         <v>0.9074093023803751</v>
       </c>
-      <c r="Q7" s="6" t="n">
-        <v>0.08626644425608526</v>
-      </c>
-      <c r="R7" s="6" t="n">
+      <c r="Q7" s="7" t="n">
+        <v>2.928193563361787</v>
+      </c>
+      <c r="R7" s="7" t="n">
         <v>0.8826984323039108</v>
       </c>
-      <c r="S7" s="6" t="n">
+      <c r="S7" s="7" t="n">
         <v>1.73440542678647</v>
       </c>
-      <c r="T7" s="6" t="n">
+      <c r="T7" s="7" t="n">
         <v>1.018645097143547</v>
       </c>
-      <c r="U7" s="6" t="n">
-        <v>-0.1492762544246609</v>
-      </c>
-      <c r="V7" s="6" t="n">
+      <c r="U7" s="7" t="n">
+        <v>3.008162184466358</v>
+      </c>
+      <c r="V7" s="7" t="n">
         <v>0.8794949403150508</v>
       </c>
-      <c r="W7" s="6" t="n">
+      <c r="W7" s="7" t="n">
         <v>1.796086583564779</v>
       </c>
-      <c r="X7" s="6" t="n">
+      <c r="X7" s="7" t="n">
         <v>0.9402443667337349</v>
       </c>
-      <c r="Y7" s="6" t="n">
-        <v>0.07764548018100573</v>
-      </c>
-      <c r="Z7" s="6" t="n">
+      <c r="Y7" s="7" t="n">
+        <v>3.225927015661399</v>
+      </c>
+      <c r="Z7" s="7" t="n">
         <v>0.8707714199822877</v>
       </c>
-      <c r="AA7" s="6" t="n">
+      <c r="AA7" s="7" t="n">
         <v>2.021870096197957</v>
       </c>
-      <c r="AB7" s="6" t="n">
+      <c r="AB7" s="7" t="n">
         <v>1.218958251398934</v>
       </c>
-      <c r="AC7" s="6" t="n">
-        <v>-0.6072625581854244</v>
-      </c>
-      <c r="AD7" s="6" t="n">
+      <c r="AC7" s="7" t="n">
+        <v>4.087958685899534</v>
+      </c>
+      <c r="AD7" s="7" t="n">
         <v>0.8362389807378955</v>
       </c>
-      <c r="AE7" s="6" t="n">
+      <c r="AE7" s="7" t="n">
         <v>1.797943155661529</v>
       </c>
-      <c r="AF7" s="6" t="n">
+      <c r="AF7" s="7" t="n">
         <v>1.024029510717094</v>
       </c>
-      <c r="AG7" s="6" t="n">
-        <v>-0.06380958392640602</v>
-      </c>
-      <c r="AH7" s="6" t="n">
+      <c r="AG7" s="7" t="n">
+        <v>3.232599590990136</v>
+      </c>
+      <c r="AH7" s="7" t="n">
         <v>0.8705041208677673</v>
       </c>
-      <c r="AI7" s="6" t="n">
+      <c r="AI7" s="7" t="n">
         <v>1.934467384061502</v>
       </c>
-      <c r="AJ7" s="6" t="n">
+      <c r="AJ7" s="7" t="n">
         <v>1.024348697447111</v>
       </c>
-      <c r="AK7" s="6" t="n">
-        <v>-0.157463065984668</v>
-      </c>
-      <c r="AL7" s="6" t="n">
+      <c r="AK7" s="7" t="n">
+        <v>3.74216405999775</v>
+      </c>
+      <c r="AL7" s="7" t="n">
         <v>0.8500912930394748</v>
       </c>
-      <c r="AM7" s="6" t="n">
+      <c r="AM7" s="7" t="n">
         <v>1.757080709068191</v>
       </c>
-      <c r="AN7" s="6" t="n">
+      <c r="AN7" s="7" t="n">
         <v>0.9216251845807225</v>
       </c>
-      <c r="AO7" s="6" t="n">
-        <v>0.1078235588733711</v>
-      </c>
-      <c r="AP7" s="6" t="n">
+      <c r="AO7" s="7" t="n">
+        <v>3.087332618179575</v>
+      </c>
+      <c r="AP7" s="7" t="n">
         <v>0.876323423204318</v>
       </c>
-      <c r="AQ7" s="6" t="n">
+      <c r="AQ7" s="7" t="n">
         <v>1.768780977731884</v>
       </c>
-      <c r="AR7" s="6" t="n">
+      <c r="AR7" s="7" t="n">
         <v>0.9288582299661345</v>
       </c>
-      <c r="AS7" s="6" t="n">
-        <v>-0.00804489189734668</v>
-      </c>
-      <c r="AT7" s="6" t="n">
+      <c r="AS7" s="7" t="n">
+        <v>3.128586147186159</v>
+      </c>
+      <c r="AT7" s="7" t="n">
         <v>0.8746708331276181</v>
       </c>
-      <c r="AU7" s="6" t="n">
+      <c r="AU7" s="7" t="n">
         <v>1.85694898820214</v>
       </c>
-      <c r="AV7" s="6" t="n">
+      <c r="AV7" s="7" t="n">
         <v>1.008833316973156</v>
       </c>
-      <c r="AW7" s="6" t="n">
-        <v>-0.2999043414160111</v>
-      </c>
-      <c r="AX7" s="6" t="n">
+      <c r="AW7" s="7" t="n">
+        <v>3.44825954478495</v>
+      </c>
+      <c r="AX7" s="7" t="n">
         <v>0.8618649205819928</v>
       </c>
-      <c r="AY7" s="6" t="n">
+      <c r="AY7" s="7" t="n">
         <v>1.79991999108792</v>
       </c>
-      <c r="AZ7" s="6" t="n">
+      <c r="AZ7" s="7" t="n">
         <v>1.035239950102736</v>
       </c>
-      <c r="BA7" s="5" t="n">
-        <v>-0.007953731252571237</v>
-      </c>
-      <c r="BB7" s="6" t="n">
+      <c r="BA7" s="7" t="n">
+        <v>3.239711974317939</v>
+      </c>
+      <c r="BB7" s="7" t="n">
         <v>0.870219203325141</v>
       </c>
-      <c r="BC7" s="6" t="n">
-        <v>1.699588758774963</v>
-      </c>
-      <c r="BD7" s="6" t="n">
-        <v>0.9045775740390447</v>
-      </c>
-      <c r="BE7" s="6" t="n">
-        <v>-0.1859068658015765</v>
-      </c>
-      <c r="BF7" s="6" t="n">
-        <v>0.8842844471410908</v>
-      </c>
-      <c r="BG7" s="5" t="n">
-        <v>1.650604119996039</v>
-      </c>
-      <c r="BH7" s="5" t="n">
-        <v>0.8615560993784805</v>
-      </c>
-      <c r="BI7" s="6" t="n">
-        <v>-0.1397272135055206</v>
-      </c>
-      <c r="BJ7" s="5" t="n">
-        <v>0.8908585085369816</v>
-      </c>
-      <c r="BK7" s="6" t="n">
+      <c r="BC7" s="7" t="n">
+        <v>1.706811649078361</v>
+      </c>
+      <c r="BD7" s="7" t="n">
+        <v>0.9237160114290024</v>
+      </c>
+      <c r="BE7" s="7" t="n">
+        <v>2.913206005429595</v>
+      </c>
+      <c r="BF7" s="7" t="n">
+        <v>0.8832988243214943</v>
+      </c>
+      <c r="BG7" s="7" t="n">
+        <v>1.69373077063702</v>
+      </c>
+      <c r="BH7" s="7" t="n">
+        <v>0.9025335527996743</v>
+      </c>
+      <c r="BI7" s="7" t="n">
+        <v>2.868723923402674</v>
+      </c>
+      <c r="BJ7" s="7" t="n">
+        <v>0.8850807481742855</v>
+      </c>
+      <c r="BK7" s="7" t="n">
         <v>1.781496294753028</v>
       </c>
-      <c r="BL7" s="6" t="n">
+      <c r="BL7" s="7" t="n">
         <v>1.121292466000662</v>
       </c>
-      <c r="BM7" s="6" t="n">
-        <v>-0.05936005570654967</v>
-      </c>
-      <c r="BN7" s="6" t="n">
+      <c r="BM7" s="7" t="n">
+        <v>3.173729048218769</v>
+      </c>
+      <c r="BN7" s="7" t="n">
         <v>0.8728624372866699</v>
       </c>
-      <c r="BO7" s="6" t="n">
+      <c r="BO7" s="7" t="n">
         <v>3.817198336140044</v>
       </c>
-      <c r="BP7" s="6" t="n">
+      <c r="BP7" s="7" t="n">
         <v>2.260349179112795</v>
       </c>
       <c r="BQ7" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="BR7" s="6" t="n">
+        <v>14.57100313743032</v>
+      </c>
+      <c r="BR7" s="7" t="n">
         <v>0.4162949019794583</v>
       </c>
-      <c r="BS7" s="6" t="n">
+      <c r="BS7" s="7" t="n">
         <v>2.72174332502565</v>
       </c>
-      <c r="BT7" s="6" t="n">
+      <c r="BT7" s="7" t="n">
         <v>1.291281341910004</v>
       </c>
-      <c r="BU7" s="6" t="n">
-        <v>-0.02107903287962768</v>
-      </c>
-      <c r="BV7" s="6" t="n">
+      <c r="BU7" s="7" t="n">
+        <v>7.407886727321683</v>
+      </c>
+      <c r="BV7" s="7" t="n">
         <v>0.7032447795451549</v>
       </c>
     </row>
@@ -1808,220 +1808,220 @@
           <t>L96-H16</t>
         </is>
       </c>
-      <c r="C8" s="7" t="n">
+      <c r="C8" s="5" t="n">
         <v>1.843530815043073</v>
       </c>
-      <c r="D8" s="7" t="n">
+      <c r="D8" s="6" t="n">
         <v>0.8524685841844074</v>
       </c>
-      <c r="E8" s="6" t="n">
-        <v>-0.03378539430967158</v>
-      </c>
-      <c r="F8" s="7" t="n">
+      <c r="E8" s="5" t="n">
+        <v>3.398605866013376</v>
+      </c>
+      <c r="F8" s="5" t="n">
         <v>0.891846579699746</v>
       </c>
-      <c r="G8" s="5" t="n">
-        <v>1.851630073606664</v>
+      <c r="G8" s="6" t="n">
+        <v>1.840209578451398</v>
       </c>
       <c r="H8" s="5" t="n">
-        <v>0.8660419602713155</v>
+        <v>0.8681533495338298</v>
       </c>
       <c r="I8" s="6" t="n">
-        <v>0.1248037177512649</v>
-      </c>
-      <c r="J8" s="5" t="n">
-        <v>0.8908941825831087</v>
-      </c>
-      <c r="K8" s="6" t="n">
+        <v>3.386371292624271</v>
+      </c>
+      <c r="J8" s="6" t="n">
+        <v>0.8922359190377313</v>
+      </c>
+      <c r="K8" s="7" t="n">
         <v>1.91235624010471</v>
       </c>
-      <c r="L8" s="6" t="n">
+      <c r="L8" s="7" t="n">
         <v>0.9271461222010317</v>
       </c>
-      <c r="M8" s="6" t="n">
-        <v>-0.03883809161989957</v>
-      </c>
-      <c r="N8" s="6" t="n">
+      <c r="M8" s="7" t="n">
+        <v>3.657106389067424</v>
+      </c>
+      <c r="N8" s="7" t="n">
         <v>0.8836203490569752</v>
       </c>
-      <c r="O8" s="6" t="n">
+      <c r="O8" s="7" t="n">
         <v>1.93411153310276</v>
       </c>
-      <c r="P8" s="6" t="n">
+      <c r="P8" s="7" t="n">
         <v>1.024111439278137</v>
       </c>
-      <c r="Q8" s="6" t="n">
-        <v>0.4914579311339247</v>
-      </c>
-      <c r="R8" s="6" t="n">
+      <c r="Q8" s="7" t="n">
+        <v>3.740787422481108</v>
+      </c>
+      <c r="R8" s="7" t="n">
         <v>0.8809573777285092</v>
       </c>
-      <c r="S8" s="6" t="n">
+      <c r="S8" s="7" t="n">
         <v>1.986477241533749</v>
       </c>
-      <c r="T8" s="6" t="n">
+      <c r="T8" s="7" t="n">
         <v>1.028369451806393</v>
       </c>
-      <c r="U8" s="6" t="n">
-        <v>0.2519332767862877</v>
-      </c>
-      <c r="V8" s="6" t="n">
+      <c r="U8" s="7" t="n">
+        <v>3.946091831131532</v>
+      </c>
+      <c r="V8" s="7" t="n">
         <v>0.8744240005516168</v>
       </c>
-      <c r="W8" s="6" t="n">
+      <c r="W8" s="7" t="n">
         <v>2.075487892838168</v>
       </c>
-      <c r="X8" s="6" t="n">
+      <c r="X8" s="7" t="n">
         <v>1.000730662831652</v>
       </c>
-      <c r="Y8" s="6" t="n">
-        <v>-0.08050047729252878</v>
-      </c>
-      <c r="Z8" s="6" t="n">
+      <c r="Y8" s="7" t="n">
+        <v>4.30764999331782</v>
+      </c>
+      <c r="Z8" s="7" t="n">
         <v>0.8629181792179444</v>
       </c>
-      <c r="AA8" s="6" t="n">
+      <c r="AA8" s="7" t="n">
         <v>2.118218963842573</v>
       </c>
-      <c r="AB8" s="6" t="n">
+      <c r="AB8" s="7" t="n">
         <v>1.4918953011226</v>
       </c>
-      <c r="AC8" s="6" t="n">
-        <v>0.6823583408757036</v>
-      </c>
-      <c r="AD8" s="6" t="n">
+      <c r="AC8" s="7" t="n">
+        <v>4.486851578782302</v>
+      </c>
+      <c r="AD8" s="7" t="n">
         <v>0.8572154690022564</v>
       </c>
-      <c r="AE8" s="6" t="n">
+      <c r="AE8" s="7" t="n">
         <v>1.935697722378429</v>
       </c>
-      <c r="AF8" s="6" t="n">
+      <c r="AF8" s="7" t="n">
         <v>1.082644095926302</v>
       </c>
-      <c r="AG8" s="6" t="n">
-        <v>0.3913886891068027</v>
-      </c>
-      <c r="AH8" s="6" t="n">
+      <c r="AG8" s="7" t="n">
+        <v>3.746925672421037</v>
+      </c>
+      <c r="AH8" s="7" t="n">
         <v>0.8807620409487138</v>
       </c>
-      <c r="AI8" s="6" t="n">
+      <c r="AI8" s="7" t="n">
         <v>2.293253695910011</v>
       </c>
-      <c r="AJ8" s="6" t="n">
+      <c r="AJ8" s="7" t="n">
         <v>1.249594322398005</v>
       </c>
-      <c r="AK8" s="6" t="n">
-        <v>0.2878859551964271</v>
-      </c>
-      <c r="AL8" s="6" t="n">
+      <c r="AK8" s="7" t="n">
+        <v>5.259012513804927</v>
+      </c>
+      <c r="AL8" s="7" t="n">
         <v>0.8326430856670566</v>
       </c>
-      <c r="AM8" s="6" t="n">
+      <c r="AM8" s="7" t="n">
         <v>2.085020338499997</v>
       </c>
-      <c r="AN8" s="6" t="n">
+      <c r="AN8" s="7" t="n">
         <v>0.988260606532289</v>
       </c>
-      <c r="AO8" s="6" t="n">
-        <v>-0.2530797428815763</v>
-      </c>
-      <c r="AP8" s="6" t="n">
+      <c r="AO8" s="7" t="n">
+        <v>4.34730981195864</v>
+      </c>
+      <c r="AP8" s="7" t="n">
         <v>0.8616560896425139</v>
       </c>
-      <c r="AQ8" s="6" t="n">
+      <c r="AQ8" s="7" t="n">
         <v>2.006911251269935</v>
       </c>
-      <c r="AR8" s="6" t="n">
+      <c r="AR8" s="7" t="n">
         <v>0.9520986193110091</v>
       </c>
-      <c r="AS8" s="6" t="n">
-        <v>-0.1762131213307913</v>
-      </c>
-      <c r="AT8" s="6" t="n">
+      <c r="AS8" s="7" t="n">
+        <v>4.027692770473857</v>
+      </c>
+      <c r="AT8" s="7" t="n">
         <v>0.8718272238032914</v>
       </c>
-      <c r="AU8" s="6" t="n">
+      <c r="AU8" s="7" t="n">
         <v>1.973075901199417</v>
       </c>
-      <c r="AV8" s="6" t="n">
+      <c r="AV8" s="7" t="n">
         <v>1.094389570369003</v>
       </c>
-      <c r="AW8" s="6" t="n">
-        <v>0.520899717920782</v>
-      </c>
-      <c r="AX8" s="6" t="n">
+      <c r="AW8" s="7" t="n">
+        <v>3.893028511893893</v>
+      </c>
+      <c r="AX8" s="7" t="n">
         <v>0.8761126280931113</v>
       </c>
-      <c r="AY8" s="6" t="n">
+      <c r="AY8" s="7" t="n">
         <v>2.045527286420046</v>
       </c>
-      <c r="AZ8" s="6" t="n">
+      <c r="AZ8" s="7" t="n">
         <v>1.047028519449541</v>
       </c>
-      <c r="BA8" s="6" t="n">
-        <v>0.07411936780444792</v>
-      </c>
-      <c r="BB8" s="6" t="n">
+      <c r="BA8" s="7" t="n">
+        <v>4.184181879488958</v>
+      </c>
+      <c r="BB8" s="7" t="n">
         <v>0.8668472899577775</v>
       </c>
-      <c r="BC8" s="6" t="n">
-        <v>2.281393267566011</v>
-      </c>
-      <c r="BD8" s="6" t="n">
-        <v>1.140807433884863</v>
-      </c>
-      <c r="BE8" s="6" t="n">
-        <v>0.7711893310252554</v>
-      </c>
-      <c r="BF8" s="6" t="n">
-        <v>0.8343697082380165</v>
-      </c>
-      <c r="BG8" s="6" t="n">
-        <v>1.940251765582014</v>
-      </c>
-      <c r="BH8" s="6" t="n">
-        <v>0.9651191386655593</v>
-      </c>
-      <c r="BI8" s="6" t="n">
-        <v>0.5037399007459268</v>
-      </c>
-      <c r="BJ8" s="6" t="n">
-        <v>0.8802003276439899</v>
-      </c>
-      <c r="BK8" s="6" t="n">
+      <c r="BC8" s="7" t="n">
+        <v>2.075908893643849</v>
+      </c>
+      <c r="BD8" s="7" t="n">
+        <v>0.9838475721162934</v>
+      </c>
+      <c r="BE8" s="7" t="n">
+        <v>4.309397734709628</v>
+      </c>
+      <c r="BF8" s="7" t="n">
+        <v>0.8628625610566228</v>
+      </c>
+      <c r="BG8" s="7" t="n">
+        <v>1.954733908096407</v>
+      </c>
+      <c r="BH8" s="7" t="n">
+        <v>0.9313905119245324</v>
+      </c>
+      <c r="BI8" s="7" t="n">
+        <v>3.820984651461852</v>
+      </c>
+      <c r="BJ8" s="7" t="n">
+        <v>0.8784052710839562</v>
+      </c>
+      <c r="BK8" s="7" t="n">
         <v>1.994858286325982</v>
       </c>
-      <c r="BL8" s="6" t="n">
+      <c r="BL8" s="7" t="n">
         <v>1.023624873050964</v>
       </c>
-      <c r="BM8" s="6" t="n">
-        <v>0.0781316295896993</v>
-      </c>
-      <c r="BN8" s="6" t="n">
+      <c r="BM8" s="7" t="n">
+        <v>3.979459582523432</v>
+      </c>
+      <c r="BN8" s="7" t="n">
         <v>0.8733621426654608</v>
       </c>
-      <c r="BO8" s="6" t="n">
+      <c r="BO8" s="7" t="n">
         <v>4.691632625905814</v>
       </c>
-      <c r="BP8" s="6" t="n">
+      <c r="BP8" s="7" t="n">
         <v>2.470033583287996</v>
       </c>
       <c r="BQ8" s="7" t="n">
-        <v>-0.003165721506897611</v>
-      </c>
-      <c r="BR8" s="6" t="n">
+        <v>22.01141669646388</v>
+      </c>
+      <c r="BR8" s="7" t="n">
         <v>0.2995333689077685</v>
       </c>
-      <c r="BS8" s="6" t="n">
+      <c r="BS8" s="7" t="n">
         <v>3.218547094750466</v>
       </c>
-      <c r="BT8" s="6" t="n">
+      <c r="BT8" s="7" t="n">
         <v>1.387438764639074</v>
       </c>
-      <c r="BU8" s="5" t="n">
-        <v>0.01434244957041818</v>
-      </c>
-      <c r="BV8" s="6" t="n">
+      <c r="BU8" s="7" t="n">
+        <v>10.35904540112666</v>
+      </c>
+      <c r="BV8" s="7" t="n">
         <v>0.6703453606135054</v>
       </c>
     </row>
@@ -2716,7 +2716,7 @@
     <row r="14" ht="48" customHeight="1">
       <c r="A14" s="9" t="inlineStr">
         <is>
-          <t>LSTM</t>
+          <t>LSTM (h128, 3L, d0.3)</t>
         </is>
       </c>
       <c r="B14" s="9" t="inlineStr">
@@ -2734,7 +2734,7 @@
       </c>
       <c r="E14" s="10" t="inlineStr">
         <is>
-          <t>public_configuration</t>
+          <t>locked_sensitivity_configuration</t>
         </is>
       </c>
       <c r="F14" s="9" t="n">
@@ -2758,13 +2758,13 @@
         <v>10</v>
       </c>
       <c r="L14" s="9" t="n">
-        <v>13.00192889999971</v>
+        <v>16.06824729999062</v>
       </c>
     </row>
     <row r="15" ht="48" customHeight="1">
       <c r="A15" s="9" t="inlineStr">
         <is>
-          <t>GRU</t>
+          <t>GRU (h64, 3L, d0.3)</t>
         </is>
       </c>
       <c r="B15" s="9" t="inlineStr">
@@ -2782,17 +2782,17 @@
       </c>
       <c r="E15" s="10" t="inlineStr">
         <is>
-          <t>public_configuration</t>
+          <t>locked_sensitivity_configuration</t>
         </is>
       </c>
       <c r="F15" s="9" t="n">
         <v>100</v>
       </c>
       <c r="G15" s="9" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="H15" s="9" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="I15" s="9" t="b">
         <v>1</v>
@@ -2806,7 +2806,7 @@
         <v>10</v>
       </c>
       <c r="L15" s="9" t="n">
-        <v>15.72156869999981</v>
+        <v>11.83939320000354</v>
       </c>
     </row>
     <row r="16" ht="48" customHeight="1">
@@ -2974,26 +2974,28 @@
       </c>
       <c r="E19" s="10" t="inlineStr">
         <is>
-          <t>Validation locked: prior=skew_b+0.50; source=round2; lr=0.0003; epsilon_c=0.5; wd=0.001; huber_beta_std=0.03238818049430847; lambda_energy=0.01; lambda_smooth=0.01; alpha*=1.0. Single test unblinding; shuffled RMSE=0.2909526453715744; no test reselection.</t>
+          <t>Validation locked: prior=skew_b+0.50; source=round2; lr=0.0003; epsilon_c=0.5; wd=0.001; huber_beta_std=0.03238818049430847; lambda_energy=0.01; lambda_smooth=0.01; alpha*=1.0. Adapter trained up to 100 epochs (patience 10) on development data, then frozen; single test unblinding; shuffled RMSE=0.2909526453715744; no test reselection.</t>
         </is>
       </c>
       <c r="F19" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="G19" s="9" t="n"/>
+        <v>100</v>
+      </c>
+      <c r="G19" s="9" t="n">
+        <v>31</v>
+      </c>
       <c r="H19" s="9" t="n">
-        <v>0</v>
+        <v>41</v>
       </c>
       <c r="I19" s="9" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J19" s="9" t="inlineStr">
         <is>
-          <t>frozen_adapter</t>
+          <t>patience</t>
         </is>
       </c>
       <c r="K19" s="9" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="L19" s="9" t="n"/>
     </row>
@@ -3576,7 +3578,7 @@
     <row r="32" ht="48" customHeight="1">
       <c r="A32" s="9" t="inlineStr">
         <is>
-          <t>LSTM</t>
+          <t>LSTM (h128, 3L, d0.3)</t>
         </is>
       </c>
       <c r="B32" s="9" t="inlineStr">
@@ -3594,17 +3596,17 @@
       </c>
       <c r="E32" s="10" t="inlineStr">
         <is>
-          <t>public_configuration</t>
+          <t>locked_sensitivity_configuration</t>
         </is>
       </c>
       <c r="F32" s="9" t="n">
         <v>100</v>
       </c>
       <c r="G32" s="9" t="n">
-        <v>17</v>
+        <v>8</v>
       </c>
       <c r="H32" s="9" t="n">
-        <v>27</v>
+        <v>18</v>
       </c>
       <c r="I32" s="9" t="b">
         <v>1</v>
@@ -3618,13 +3620,13 @@
         <v>10</v>
       </c>
       <c r="L32" s="9" t="n">
-        <v>14.52299230000062</v>
+        <v>18.60896800001501</v>
       </c>
     </row>
     <row r="33" ht="48" customHeight="1">
       <c r="A33" s="9" t="inlineStr">
         <is>
-          <t>GRU</t>
+          <t>GRU (h64, 3L, d0.3)</t>
         </is>
       </c>
       <c r="B33" s="9" t="inlineStr">
@@ -3642,17 +3644,17 @@
       </c>
       <c r="E33" s="10" t="inlineStr">
         <is>
-          <t>public_configuration</t>
+          <t>locked_sensitivity_configuration</t>
         </is>
       </c>
       <c r="F33" s="9" t="n">
         <v>100</v>
       </c>
       <c r="G33" s="9" t="n">
-        <v>42</v>
+        <v>22</v>
       </c>
       <c r="H33" s="9" t="n">
-        <v>52</v>
+        <v>32</v>
       </c>
       <c r="I33" s="9" t="b">
         <v>1</v>
@@ -3666,7 +3668,7 @@
         <v>10</v>
       </c>
       <c r="L33" s="9" t="n">
-        <v>25.43186820000119</v>
+        <v>20.54262379999273</v>
       </c>
     </row>
     <row r="34" ht="48" customHeight="1">
@@ -3834,26 +3836,28 @@
       </c>
       <c r="E37" s="10" t="inlineStr">
         <is>
-          <t>Validation locked: prior=skew_b+0.50; source=round1; lr=0.0003; epsilon_c=1.0; wd=0.0; huber_beta_std=1.0; lambda_energy=0.0; lambda_smooth=0.0; alpha*=1.0. Single test unblinding; shuffled RMSE=0.7336189738013505; no test reselection.</t>
+          <t>Validation locked: prior=mean_q_full; source=round1; lr=0.0003; epsilon_c=1.0; wd=0.0; huber_beta_std=1.0; lambda_energy=0.0; lambda_smooth=0.0; alpha*=1.0. Adapter trained up to 100 epochs (patience 10) on development data, then frozen; single test unblinding; shuffled RMSE=0.7336208198147224; no test reselection.</t>
         </is>
       </c>
       <c r="F37" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="G37" s="9" t="n"/>
+        <v>100</v>
+      </c>
+      <c r="G37" s="9" t="n">
+        <v>48</v>
+      </c>
       <c r="H37" s="9" t="n">
-        <v>0</v>
+        <v>58</v>
       </c>
       <c r="I37" s="9" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J37" s="9" t="inlineStr">
         <is>
-          <t>frozen_adapter</t>
+          <t>patience</t>
         </is>
       </c>
       <c r="K37" s="9" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="L37" s="9" t="n"/>
     </row>
@@ -4436,7 +4440,7 @@
     <row r="50" ht="48" customHeight="1">
       <c r="A50" s="9" t="inlineStr">
         <is>
-          <t>LSTM</t>
+          <t>LSTM (h128, 3L, d0.3)</t>
         </is>
       </c>
       <c r="B50" s="9" t="inlineStr">
@@ -4454,17 +4458,17 @@
       </c>
       <c r="E50" s="10" t="inlineStr">
         <is>
-          <t>public_configuration</t>
+          <t>locked_sensitivity_configuration</t>
         </is>
       </c>
       <c r="F50" s="9" t="n">
         <v>100</v>
       </c>
       <c r="G50" s="9" t="n">
-        <v>14</v>
+        <v>19</v>
       </c>
       <c r="H50" s="9" t="n">
-        <v>24</v>
+        <v>29</v>
       </c>
       <c r="I50" s="9" t="b">
         <v>1</v>
@@ -4478,13 +4482,13 @@
         <v>10</v>
       </c>
       <c r="L50" s="9" t="n">
-        <v>10.37699570000041</v>
+        <v>21.54941199999303</v>
       </c>
     </row>
     <row r="51" ht="48" customHeight="1">
       <c r="A51" s="9" t="inlineStr">
         <is>
-          <t>GRU</t>
+          <t>GRU (h64, 3L, d0.3)</t>
         </is>
       </c>
       <c r="B51" s="9" t="inlineStr">
@@ -4502,7 +4506,7 @@
       </c>
       <c r="E51" s="10" t="inlineStr">
         <is>
-          <t>public_configuration</t>
+          <t>locked_sensitivity_configuration</t>
         </is>
       </c>
       <c r="F51" s="9" t="n">
@@ -4526,7 +4530,7 @@
         <v>10</v>
       </c>
       <c r="L51" s="9" t="n">
-        <v>16.72461030000341</v>
+        <v>18.40350730001228</v>
       </c>
     </row>
     <row r="52" ht="48" customHeight="1">
@@ -4694,26 +4698,28 @@
       </c>
       <c r="E55" s="10" t="inlineStr">
         <is>
-          <t>Validation locked: prior=mean_q_full; source=round1; lr=0.0003; epsilon_c=1.0; wd=0.0; huber_beta_std=1.0; lambda_energy=0.0; lambda_smooth=0.0; alpha*=1.0. Single test unblinding; shuffled RMSE=1.6539449326733247; no test reselection.</t>
+          <t>Validation locked: prior=mean_q_full; source=round1; lr=0.0003; epsilon_c=1.0; wd=0.0; huber_beta_std=1.0; lambda_energy=0.0; lambda_smooth=0.0; alpha*=1.0. Adapter trained up to 100 epochs (patience 10) on development data, then frozen; single test unblinding; shuffled RMSE=1.6539449326733247; no test reselection.</t>
         </is>
       </c>
       <c r="F55" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="G55" s="9" t="n"/>
+        <v>100</v>
+      </c>
+      <c r="G55" s="9" t="n">
+        <v>33</v>
+      </c>
       <c r="H55" s="9" t="n">
-        <v>0</v>
+        <v>43</v>
       </c>
       <c r="I55" s="9" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J55" s="9" t="inlineStr">
         <is>
-          <t>frozen_adapter</t>
+          <t>patience</t>
         </is>
       </c>
       <c r="K55" s="9" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="L55" s="9" t="n"/>
     </row>
@@ -5296,7 +5302,7 @@
     <row r="68" ht="48" customHeight="1">
       <c r="A68" s="9" t="inlineStr">
         <is>
-          <t>LSTM</t>
+          <t>LSTM (h128, 3L, d0.3)</t>
         </is>
       </c>
       <c r="B68" s="9" t="inlineStr">
@@ -5314,17 +5320,17 @@
       </c>
       <c r="E68" s="10" t="inlineStr">
         <is>
-          <t>public_configuration</t>
+          <t>locked_sensitivity_configuration</t>
         </is>
       </c>
       <c r="F68" s="9" t="n">
         <v>100</v>
       </c>
       <c r="G68" s="9" t="n">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="H68" s="9" t="n">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="I68" s="9" t="b">
         <v>1</v>
@@ -5338,13 +5344,13 @@
         <v>10</v>
       </c>
       <c r="L68" s="9" t="n">
-        <v>13.13952920000065</v>
+        <v>26.3829473000078</v>
       </c>
     </row>
     <row r="69" ht="48" customHeight="1">
       <c r="A69" s="9" t="inlineStr">
         <is>
-          <t>GRU</t>
+          <t>GRU (h64, 3L, d0.3)</t>
         </is>
       </c>
       <c r="B69" s="9" t="inlineStr">
@@ -5362,7 +5368,7 @@
       </c>
       <c r="E69" s="10" t="inlineStr">
         <is>
-          <t>public_configuration</t>
+          <t>locked_sensitivity_configuration</t>
         </is>
       </c>
       <c r="F69" s="9" t="n">
@@ -5386,7 +5392,7 @@
         <v>10</v>
       </c>
       <c r="L69" s="9" t="n">
-        <v>13.20026690000032</v>
+        <v>16.41980819997843</v>
       </c>
     </row>
     <row r="70" ht="48" customHeight="1">
@@ -5554,26 +5560,28 @@
       </c>
       <c r="E73" s="10" t="inlineStr">
         <is>
-          <t>Validation locked: prior=mean_q_full; source=round1; lr=0.0003; epsilon_c=0.5; wd=0.0; huber_beta_std=1.0; lambda_energy=0.0; lambda_smooth=0.0; alpha*=1.0. Single test unblinding; shuffled RMSE=1.853421711932899; no test reselection. FM test result is worse than PSRC and is retained as observed.</t>
+          <t>Validation locked: prior=mean_q_full; source=retune1; lr=3e-05; epsilon_c=0.25; wd=0.0; huber_beta_std=1.0; lambda_energy=0.0; lambda_smooth=0.0; alpha*=1.0. Adapter trained up to 100 epochs (patience 10) on development data, then frozen; single test unblinding; shuffled RMSE=1.8451713988011604; no test reselection. FM test result is worse than PSRC and is retained as observed.</t>
         </is>
       </c>
       <c r="F73" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="G73" s="9" t="n"/>
+        <v>100</v>
+      </c>
+      <c r="G73" s="9" t="n">
+        <v>67</v>
+      </c>
       <c r="H73" s="9" t="n">
-        <v>0</v>
+        <v>77</v>
       </c>
       <c r="I73" s="9" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J73" s="9" t="inlineStr">
         <is>
-          <t>frozen_adapter</t>
+          <t>patience</t>
         </is>
       </c>
       <c r="K73" s="9" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="L73" s="9" t="n"/>
     </row>

</xml_diff>